<commit_message>
Swap day and month in folder and file naming, New Result Wed
</commit_message>
<xml_diff>
--- a/Backtest/01-02-18/S&P500stock_01-02-18period252RS90.xlsx
+++ b/Backtest/01-02-18/S&P500stock_01-02-18period252RS90.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="82">
   <si>
     <t>Stock</t>
   </si>
@@ -127,148 +127,139 @@
     <t>EM Rating</t>
   </si>
   <si>
-    <t>TTWO</t>
+    <t>CAT</t>
+  </si>
+  <si>
+    <t>FMC</t>
+  </si>
+  <si>
+    <t>MCO</t>
+  </si>
+  <si>
+    <t>MAR</t>
+  </si>
+  <si>
+    <t>ELV</t>
   </si>
   <si>
     <t>BA</t>
   </si>
   <si>
-    <t>NOW</t>
-  </si>
-  <si>
-    <t>MAR</t>
-  </si>
-  <si>
-    <t>NTAP</t>
-  </si>
-  <si>
-    <t>NFLX</t>
-  </si>
-  <si>
-    <t>ELV</t>
-  </si>
-  <si>
-    <t>NVDA</t>
-  </si>
-  <si>
-    <t>ADBE</t>
-  </si>
-  <si>
-    <t>PYPL</t>
-  </si>
-  <si>
     <t>MSCI</t>
   </si>
   <si>
+    <t>NVR</t>
+  </si>
+  <si>
     <t>MTCH</t>
   </si>
   <si>
     <t>ANET</t>
   </si>
   <si>
+    <t>NRG</t>
+  </si>
+  <si>
     <t>PODD</t>
   </si>
   <si>
-    <t>TPL</t>
-  </si>
-  <si>
-    <t>MV</t>
+    <t>AVY</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
+    <t>2018-01-25</t>
+  </si>
+  <si>
+    <t>2018-02-12</t>
+  </si>
+  <si>
+    <t>2018-02-09</t>
+  </si>
+  <si>
+    <t>2018-02-14</t>
+  </si>
+  <si>
+    <t>2018-01-31</t>
+  </si>
+  <si>
+    <t>2018-02-01</t>
+  </si>
+  <si>
     <t>2018-02-07</t>
   </si>
   <si>
-    <t>2018-04-25</t>
-  </si>
-  <si>
-    <t>2018-02-14</t>
-  </si>
-  <si>
-    <t>2018-04-16</t>
-  </si>
-  <si>
-    <t>2018-02-08</t>
-  </si>
-  <si>
-    <t>2018-03-15</t>
-  </si>
-  <si>
-    <t>2018-05-03</t>
-  </si>
-  <si>
     <t>2018-02-15</t>
   </si>
   <si>
+    <t>2018-03-01</t>
+  </si>
+  <si>
     <t>2018-02-21</t>
   </si>
   <si>
-    <t>2018-04-30</t>
+    <t>Industrials</t>
+  </si>
+  <si>
+    <t>Basic Materials</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Consumer Cyclical</t>
+  </si>
+  <si>
+    <t>Healthcare</t>
   </si>
   <si>
     <t>Communication Services</t>
   </si>
   <si>
-    <t>Industrials</t>
-  </si>
-  <si>
     <t>Technology</t>
   </si>
   <si>
-    <t>Consumer Cyclical</t>
-  </si>
-  <si>
-    <t>Healthcare</t>
-  </si>
-  <si>
-    <t>Financial Services</t>
-  </si>
-  <si>
-    <t>Energy</t>
-  </si>
-  <si>
-    <t>Electronic Gaming &amp; Multimedia</t>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Farm &amp; Heavy Construction Machinery</t>
+  </si>
+  <si>
+    <t>Agricultural Inputs</t>
+  </si>
+  <si>
+    <t>Financial Data &amp; Stock Exchanges</t>
+  </si>
+  <si>
+    <t>Lodging</t>
+  </si>
+  <si>
+    <t>Healthcare Plans</t>
   </si>
   <si>
     <t>Aerospace &amp; Defense</t>
   </si>
   <si>
-    <t>Software - Application</t>
-  </si>
-  <si>
-    <t>Lodging</t>
+    <t>Residential Construction</t>
+  </si>
+  <si>
+    <t>Internet Content &amp; Information</t>
   </si>
   <si>
     <t>Computer Hardware</t>
   </si>
   <si>
-    <t>Entertainment</t>
-  </si>
-  <si>
-    <t>Healthcare Plans</t>
-  </si>
-  <si>
-    <t>Semiconductors</t>
-  </si>
-  <si>
-    <t>Software - Infrastructure</t>
-  </si>
-  <si>
-    <t>Credit Services</t>
-  </si>
-  <si>
-    <t>Financial Data &amp; Stock Exchanges</t>
-  </si>
-  <si>
-    <t>Internet Content &amp; Information</t>
+    <t>Utilities - Independent Power Producers</t>
   </si>
   <si>
     <t>Medical Devices</t>
   </si>
   <si>
-    <t>Oil &amp; Gas E&amp;P</t>
+    <t>Packaging &amp; Containers</t>
   </si>
 </sst>
 </file>
@@ -626,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK16"/>
+  <dimension ref="A1:AK14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:37">
@@ -747,49 +738,49 @@
         <v>37</v>
       </c>
       <c r="B2">
-        <v>99.58592132505176</v>
+        <v>94.6058091286307</v>
       </c>
       <c r="C2">
-        <v>281</v>
+        <v>123</v>
       </c>
       <c r="D2">
-        <v>126.67</v>
+        <v>157.58</v>
       </c>
       <c r="E2">
-        <v>2.01</v>
+        <v>1.12</v>
       </c>
       <c r="F2">
-        <v>0.1986543300886651</v>
+        <v>-0.2108438787796711</v>
       </c>
       <c r="G2">
-        <v>2.34</v>
+        <v>1.14</v>
       </c>
       <c r="H2">
-        <v>0.6200407014007362</v>
+        <v>-0.5454201222182009</v>
       </c>
       <c r="I2">
-        <v>120.1679992675782</v>
+        <v>157.1420013427734</v>
       </c>
       <c r="J2">
-        <v>117.2290000915527</v>
+        <v>148.6265014648438</v>
       </c>
       <c r="K2">
-        <v>113.3394000244141</v>
+        <v>141.4044006347656</v>
       </c>
       <c r="L2">
-        <v>93.54264995574951</v>
+        <v>117.0711000442505</v>
       </c>
       <c r="M2">
-        <v>1.03</v>
+        <v>1.06</v>
       </c>
       <c r="N2">
-        <v>1.06</v>
+        <v>1.11</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -798,7 +789,7 @@
         <v>0</v>
       </c>
       <c r="T2">
-        <v>4.444444444444444</v>
+        <v>2.222222222222222</v>
       </c>
       <c r="U2" t="b">
         <v>0</v>
@@ -807,49 +798,49 @@
         <v>1</v>
       </c>
       <c r="W2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2">
-        <v>53.35</v>
+        <v>90.34</v>
       </c>
       <c r="Y2">
-        <v>127.77</v>
+        <v>158.65</v>
       </c>
       <c r="Z2">
-        <v>11.19</v>
+        <v>74.84</v>
       </c>
       <c r="AA2">
-        <v>-15.04</v>
+        <v>0.24</v>
       </c>
       <c r="AB2">
-        <v>485.29</v>
+        <v>777.27</v>
       </c>
       <c r="AC2">
-        <v>90.91</v>
+        <v>189.95</v>
       </c>
       <c r="AD2">
-        <v>-0.19</v>
+        <v>6.76</v>
       </c>
       <c r="AE2">
-        <v>-105.26</v>
+        <v>31.62</v>
       </c>
       <c r="AF2">
-        <v>-48.18</v>
+        <v>312.12</v>
       </c>
       <c r="AG2">
-        <v>433.33</v>
+        <v>116.58</v>
       </c>
       <c r="AH2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="AI2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="AJ2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AK2">
-        <v>87.42733025284247</v>
+        <v>91.0719727202122</v>
       </c>
     </row>
     <row r="3" spans="1:37">
@@ -857,49 +848,52 @@
         <v>38</v>
       </c>
       <c r="B3">
-        <v>98.9648033126294</v>
+        <v>94.1908713692946</v>
       </c>
       <c r="C3">
-        <v>109</v>
+        <v>361</v>
       </c>
       <c r="D3">
-        <v>354.37</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="E3">
-        <v>2.12</v>
+        <v>1.24</v>
       </c>
       <c r="F3">
-        <v>0.3381350299381538</v>
+        <v>0.02078742466841802</v>
       </c>
       <c r="G3">
-        <v>1.47</v>
+        <v>1.15</v>
       </c>
       <c r="H3">
-        <v>-0.7064398155303466</v>
+        <v>-0.530770408191679</v>
       </c>
       <c r="I3">
-        <v>343.84599609375</v>
+        <v>82.47354736328126</v>
       </c>
       <c r="J3">
-        <v>330.4024993896484</v>
+        <v>80.0867301940918</v>
       </c>
       <c r="K3">
-        <v>301.9383990478516</v>
+        <v>80.50702545166016</v>
       </c>
       <c r="L3">
-        <v>242.989800491333</v>
+        <v>71.17662603378295</v>
       </c>
       <c r="M3">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="N3">
-        <v>1.14</v>
+        <v>1.02</v>
+      </c>
+      <c r="O3" t="s">
+        <v>50</v>
       </c>
       <c r="P3">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="Q3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -908,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="T3">
-        <v>15</v>
+        <v>2.222222222222222</v>
       </c>
       <c r="U3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
@@ -920,46 +914,46 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>160.82</v>
+        <v>48.87</v>
       </c>
       <c r="Y3">
-        <v>360.97</v>
+        <v>83.28</v>
       </c>
       <c r="Z3">
-        <v>179.9</v>
+        <v>10.53</v>
       </c>
       <c r="AA3">
-        <v>6.44</v>
+        <v>0.25</v>
       </c>
       <c r="AB3">
-        <v>33.75</v>
+        <v>220</v>
       </c>
       <c r="AC3">
-        <v>114.79</v>
+        <v>241.67</v>
       </c>
       <c r="AD3">
-        <v>193.81</v>
+        <v>3.32</v>
       </c>
       <c r="AE3">
-        <v>82.18000000000001</v>
+        <v>-26.79</v>
       </c>
       <c r="AF3">
-        <v>4.12</v>
+        <v>160.22</v>
       </c>
       <c r="AG3">
-        <v>13.23</v>
+        <v>-875</v>
       </c>
       <c r="AH3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="AI3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="AJ3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AK3">
-        <v>72.54896324183559</v>
+        <v>80.87206734059239</v>
       </c>
     </row>
     <row r="4" spans="1:37">
@@ -967,52 +961,49 @@
         <v>39</v>
       </c>
       <c r="B4">
-        <v>91.92546583850931</v>
+        <v>90.87136929460581</v>
       </c>
       <c r="C4">
-        <v>272</v>
+        <v>402</v>
       </c>
       <c r="D4">
-        <v>148.87</v>
+        <v>147.61</v>
       </c>
       <c r="E4">
-        <v>0.87</v>
+        <v>0.6</v>
       </c>
       <c r="F4">
-        <v>-1.24687292289694</v>
+        <v>-1.214579527054725</v>
       </c>
       <c r="G4">
-        <v>1.6</v>
+        <v>0.82</v>
       </c>
       <c r="H4">
-        <v>-0.508230083115357</v>
+        <v>-1.014210971066902</v>
       </c>
       <c r="I4">
-        <v>147.5659973144531</v>
+        <v>146.9840026855469</v>
       </c>
       <c r="J4">
-        <v>141.0049987792969</v>
+        <v>149.9105010986328</v>
       </c>
       <c r="K4">
-        <v>131.8545997619629</v>
+        <v>147.512200012207</v>
       </c>
       <c r="L4">
-        <v>115.5440501403809</v>
+        <v>130.5681003189087</v>
       </c>
       <c r="M4">
-        <v>1.05</v>
+        <v>0.98</v>
       </c>
       <c r="N4">
-        <v>1.12</v>
-      </c>
-      <c r="O4" t="s">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="P4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -1021,58 +1012,58 @@
         <v>0</v>
       </c>
       <c r="T4">
-        <v>12.77777777777778</v>
+        <v>6.11111111111111</v>
       </c>
       <c r="U4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X4">
-        <v>83.42</v>
+        <v>93.51000000000001</v>
       </c>
       <c r="Y4">
-        <v>150.85</v>
+        <v>153.86</v>
       </c>
       <c r="Z4">
-        <v>22.32</v>
+        <v>27.02</v>
       </c>
       <c r="AA4">
-        <v>36.55</v>
+        <v>4.65</v>
       </c>
       <c r="AB4">
-        <v>74.34</v>
+        <v>16.13</v>
       </c>
       <c r="AC4">
-        <v>30.77</v>
+        <v>174.77</v>
       </c>
       <c r="AD4">
-        <v>-2.23</v>
+        <v>-203.89</v>
       </c>
       <c r="AE4">
-        <v>30.77</v>
+        <v>1.84</v>
       </c>
       <c r="AF4">
-        <v>60.61</v>
+        <v>-9.94</v>
       </c>
       <c r="AG4">
-        <v>-153.85</v>
+        <v>181.53</v>
       </c>
       <c r="AH4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AI4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="AJ4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AK4">
-        <v>63.37622363889784</v>
+        <v>57.85589088859231</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -1080,49 +1071,49 @@
         <v>40</v>
       </c>
       <c r="B5">
-        <v>95.65217391304348</v>
+        <v>93.3609958506224</v>
       </c>
       <c r="C5">
-        <v>301</v>
+        <v>168</v>
       </c>
       <c r="D5">
-        <v>147.34</v>
+        <v>135.73</v>
       </c>
       <c r="E5">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="F5">
-        <v>-1.056671968556729</v>
+        <v>-0.5775934425724792</v>
       </c>
       <c r="G5">
-        <v>0.98</v>
+        <v>0.88</v>
       </c>
       <c r="H5">
-        <v>-1.453538037709922</v>
+        <v>-0.9263126869077706</v>
       </c>
       <c r="I5">
-        <v>147.0480010986328</v>
+        <v>135.1640014648438</v>
       </c>
       <c r="J5">
-        <v>141.6534996032715</v>
+        <v>131.0010009765625</v>
       </c>
       <c r="K5">
-        <v>134.5212004089356</v>
+        <v>125.3360005187988</v>
       </c>
       <c r="L5">
-        <v>112.9098998641968</v>
+        <v>107.744949836731</v>
       </c>
       <c r="M5">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="N5">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -1131,7 +1122,7 @@
         <v>0</v>
       </c>
       <c r="T5">
-        <v>0</v>
+        <v>2.777777777777778</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -1143,10 +1134,10 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>83.81</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="Y5">
-        <v>149.21</v>
+        <v>137.6</v>
       </c>
       <c r="Z5">
         <v>41.52</v>
@@ -1173,16 +1164,16 @@
         <v>39.13</v>
       </c>
       <c r="AH5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AI5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AJ5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AK5">
-        <v>54.31718559290773</v>
+        <v>46.62288664575777</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -1190,46 +1181,46 @@
         <v>41</v>
       </c>
       <c r="B6">
-        <v>90.06211180124224</v>
+        <v>90.04149377593362</v>
       </c>
       <c r="C6">
-        <v>225</v>
+        <v>304</v>
       </c>
       <c r="D6">
-        <v>61.5</v>
+        <v>225.01</v>
       </c>
       <c r="E6">
-        <v>1.28</v>
+        <v>1.11</v>
       </c>
       <c r="F6">
-        <v>-0.7269903143670291</v>
+        <v>-0.2301464874003452</v>
       </c>
       <c r="G6">
-        <v>2.31</v>
+        <v>1.33</v>
       </c>
       <c r="H6">
-        <v>0.5742999939203544</v>
+        <v>-0.2670755557142842</v>
       </c>
       <c r="I6">
-        <v>62.48800048828125</v>
+        <v>225.6639984130859</v>
       </c>
       <c r="J6">
-        <v>61.66300029754639</v>
+        <v>226.4235008239746</v>
       </c>
       <c r="K6">
-        <v>58.56839996337891</v>
+        <v>218.968600769043</v>
       </c>
       <c r="L6">
-        <v>45.78719997406006</v>
+        <v>192.7488004302978</v>
       </c>
       <c r="M6">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="N6">
-        <v>1.07</v>
+        <v>1.03</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
         <v>1</v>
@@ -1241,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="T6">
-        <v>1.111111111111111</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="U6" t="b">
         <v>1</v>
@@ -1253,34 +1244,34 @@
         <v>1</v>
       </c>
       <c r="X6">
-        <v>37.43</v>
+        <v>140.5</v>
       </c>
       <c r="Y6">
-        <v>64.06</v>
+        <v>236.39</v>
       </c>
       <c r="Z6">
-        <v>12.22</v>
+        <v>50.7</v>
       </c>
       <c r="AA6">
-        <v>15.17</v>
+        <v>2.62</v>
       </c>
       <c r="AB6">
-        <v>38.41</v>
+        <v>11.99</v>
       </c>
       <c r="AC6">
-        <v>22.64</v>
+        <v>107.97</v>
       </c>
       <c r="AD6">
-        <v>6.27</v>
+        <v>2.88</v>
       </c>
       <c r="AE6">
-        <v>32.65</v>
+        <v>-11.15</v>
       </c>
       <c r="AF6">
-        <v>-18.33</v>
+        <v>-15.45</v>
       </c>
       <c r="AG6">
-        <v>13.21</v>
+        <v>176.81</v>
       </c>
       <c r="AH6" t="s">
         <v>56</v>
@@ -1289,10 +1280,10 @@
         <v>66</v>
       </c>
       <c r="AJ6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AK6">
-        <v>46.15782346184089</v>
+        <v>42.66304214118399</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -1300,49 +1291,49 @@
         <v>42</v>
       </c>
       <c r="B7">
-        <v>97.51552795031056</v>
+        <v>97.71784232365145</v>
       </c>
       <c r="C7">
-        <v>36</v>
+        <v>193</v>
       </c>
       <c r="D7">
-        <v>270.3</v>
+        <v>294.91</v>
       </c>
       <c r="E7">
-        <v>2.81</v>
+        <v>1.09</v>
       </c>
       <c r="F7">
-        <v>1.213059419903125</v>
+        <v>-0.2687517046416935</v>
       </c>
       <c r="G7">
-        <v>2.2</v>
+        <v>1.02</v>
       </c>
       <c r="H7">
-        <v>0.4065840664922866</v>
+        <v>-0.7212166905364638</v>
       </c>
       <c r="I7">
-        <v>275.597998046875</v>
+        <v>295.4679992675781</v>
       </c>
       <c r="J7">
-        <v>234.5</v>
+        <v>289.3725006103516</v>
       </c>
       <c r="K7">
-        <v>207.8744003295898</v>
+        <v>273.7692010498047</v>
       </c>
       <c r="L7">
-        <v>181.2786499786377</v>
+        <v>227.0999006652832</v>
       </c>
       <c r="M7">
-        <v>1.18</v>
+        <v>1.02</v>
       </c>
       <c r="N7">
-        <v>1.33</v>
+        <v>1.08</v>
       </c>
       <c r="O7" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q7">
         <v>2</v>
@@ -1351,61 +1342,61 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T7">
-        <v>13.88888888888889</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="U7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" t="b">
         <v>1</v>
       </c>
       <c r="X7">
-        <v>138.26</v>
+        <v>154.96</v>
       </c>
       <c r="Y7">
-        <v>286.81</v>
+        <v>299.33</v>
       </c>
       <c r="Z7">
-        <v>85.77</v>
+        <v>154.13</v>
       </c>
       <c r="AA7">
-        <v>9765.48</v>
+        <v>4.6</v>
       </c>
       <c r="AB7">
-        <v>51.76</v>
+        <v>19.81</v>
       </c>
       <c r="AC7">
-        <v>4.88</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="AD7">
-        <v>5.18</v>
+        <v>158.08</v>
       </c>
       <c r="AE7">
-        <v>43.33</v>
+        <v>4.12</v>
       </c>
       <c r="AF7">
-        <v>100</v>
+        <v>13.23</v>
       </c>
       <c r="AG7">
-        <v>-63.41</v>
+        <v>-8.210000000000001</v>
       </c>
       <c r="AH7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AI7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="AJ7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AK7">
-        <v>41.36434502300899</v>
+        <v>27.37052817407087</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -1413,49 +1404,49 @@
         <v>43</v>
       </c>
       <c r="B8">
-        <v>90.26915113871635</v>
+        <v>92.53112033195021</v>
       </c>
       <c r="C8">
-        <v>224</v>
+        <v>423</v>
       </c>
       <c r="D8">
-        <v>247.85</v>
+        <v>126.54</v>
       </c>
       <c r="E8">
-        <v>1.75</v>
+        <v>0.68</v>
       </c>
       <c r="F8">
-        <v>-0.131027324101034</v>
+        <v>-1.060158658089332</v>
       </c>
       <c r="G8">
-        <v>1.36</v>
+        <v>1.18</v>
       </c>
       <c r="H8">
-        <v>-0.8741557429584144</v>
+        <v>-0.4868212661121131</v>
       </c>
       <c r="I8">
-        <v>251.5700012207031</v>
+        <v>126.4639999389648</v>
       </c>
       <c r="J8">
-        <v>243.567000579834</v>
+        <v>127.5630001068115</v>
       </c>
       <c r="K8">
-        <v>232.6310006713867</v>
+        <v>125.7265998840332</v>
       </c>
       <c r="L8">
-        <v>200.8155004119873</v>
+        <v>111.2925999832153</v>
       </c>
       <c r="M8">
-        <v>1.03</v>
+        <v>0.99</v>
       </c>
       <c r="N8">
-        <v>1.08</v>
+        <v>1.01</v>
       </c>
       <c r="P8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <v>0</v>
@@ -1464,58 +1455,58 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>5</v>
+        <v>1.111111111111111</v>
       </c>
       <c r="U8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" t="b">
         <v>0</v>
       </c>
       <c r="W8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X8">
-        <v>154.37</v>
+        <v>78.34999999999999</v>
       </c>
       <c r="Y8">
-        <v>267.95</v>
+        <v>130.58</v>
       </c>
       <c r="Z8">
-        <v>60.26</v>
+        <v>10.74</v>
       </c>
       <c r="AA8">
-        <v>2.35</v>
+        <v>19.48</v>
       </c>
       <c r="AB8">
-        <v>11.28</v>
+        <v>2.43</v>
       </c>
       <c r="AC8">
-        <v>25.13</v>
+        <v>28.77</v>
       </c>
       <c r="AD8">
-        <v>4.64</v>
+        <v>23.63</v>
       </c>
       <c r="AE8">
-        <v>66.55</v>
+        <v>4.44</v>
       </c>
       <c r="AF8">
-        <v>-11.15</v>
+        <v>12.5</v>
       </c>
       <c r="AG8">
-        <v>-15.45</v>
+        <v>9.59</v>
       </c>
       <c r="AH8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AI8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="AJ8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AK8">
-        <v>39.04350455503288</v>
+        <v>14.3700671402518</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -1523,43 +1514,43 @@
         <v>44</v>
       </c>
       <c r="B9">
-        <v>99.37888198757764</v>
+        <v>98.96265560165975</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>481</v>
       </c>
       <c r="D9">
-        <v>6.14</v>
+        <v>3508.22</v>
       </c>
       <c r="E9">
-        <v>1.9</v>
+        <v>0.98</v>
       </c>
       <c r="F9">
-        <v>0.05917363023917706</v>
+        <v>-0.4810803994691089</v>
       </c>
       <c r="G9">
-        <v>2.14</v>
+        <v>1.45</v>
       </c>
       <c r="H9">
-        <v>0.3151026515315221</v>
+        <v>-0.09127898739602132</v>
       </c>
       <c r="I9">
-        <v>6.07524995803833</v>
+        <v>3489.389990234375</v>
       </c>
       <c r="J9">
-        <v>5.723712515830994</v>
+        <v>3430.469482421875</v>
       </c>
       <c r="K9">
-        <v>5.26784499168396</v>
+        <v>3345.260185546875</v>
       </c>
       <c r="L9">
-        <v>4.347144991159439</v>
+        <v>2692.856045532227</v>
       </c>
       <c r="M9">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="N9">
-        <v>1.15</v>
+        <v>1.04</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1577,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="U9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="b">
         <v>1</v>
@@ -1586,46 +1577,46 @@
         <v>1</v>
       </c>
       <c r="X9">
-        <v>2.38</v>
+        <v>1631.78</v>
       </c>
       <c r="Y9">
-        <v>6.23</v>
+        <v>3536.97</v>
       </c>
       <c r="Z9">
-        <v>129.88</v>
+        <v>12.17</v>
       </c>
       <c r="AA9">
-        <v>2903.8</v>
+        <v>1.68</v>
       </c>
       <c r="AB9">
-        <v>27.27</v>
+        <v>4.08</v>
       </c>
       <c r="AC9">
-        <v>16.78</v>
+        <v>8.75</v>
       </c>
       <c r="AD9">
-        <v>13.19</v>
+        <v>9.82</v>
       </c>
       <c r="AE9">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="AF9">
         <v>42.04</v>
       </c>
-      <c r="AF9">
-        <v>13.95</v>
-      </c>
       <c r="AG9">
-        <v>-27.85</v>
+        <v>-30.17</v>
       </c>
       <c r="AH9" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="AI9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AJ9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="AK9">
-        <v>39.04103678613745</v>
+        <v>4.591751550201111</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -1633,49 +1624,49 @@
         <v>45</v>
       </c>
       <c r="B10">
-        <v>95.8592132505176</v>
+        <v>96.6804979253112</v>
       </c>
       <c r="C10">
-        <v>223</v>
+        <v>285</v>
       </c>
       <c r="D10">
-        <v>199.76</v>
+        <v>31.31</v>
       </c>
       <c r="E10">
-        <v>1.26</v>
+        <v>1.86</v>
       </c>
       <c r="F10">
-        <v>-0.7523504416123906</v>
+        <v>1.217549159150213</v>
       </c>
       <c r="G10">
-        <v>1.55</v>
+        <v>2.27</v>
       </c>
       <c r="H10">
-        <v>-0.5844645955826607</v>
+        <v>1.109997562778776</v>
       </c>
       <c r="I10">
-        <v>198.7399963378906</v>
+        <v>31.56599998474121</v>
       </c>
       <c r="J10">
-        <v>193.135498046875</v>
+        <v>29.99000005722046</v>
       </c>
       <c r="K10">
-        <v>183.4943994140625</v>
+        <v>28.74719989776611</v>
       </c>
       <c r="L10">
-        <v>158.0417501831055</v>
+        <v>21.85247493743897</v>
       </c>
       <c r="M10">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="N10">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R10">
         <v>0</v>
@@ -1684,58 +1675,58 @@
         <v>0</v>
       </c>
       <c r="T10">
-        <v>1.111111111111111</v>
+        <v>0</v>
       </c>
       <c r="U10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V10" t="b">
         <v>1</v>
       </c>
       <c r="W10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10">
-        <v>112.27</v>
+        <v>15.42</v>
       </c>
       <c r="Y10">
-        <v>204.45</v>
+        <v>32.87</v>
       </c>
       <c r="Z10">
-        <v>90.94</v>
+        <v>2.02</v>
       </c>
       <c r="AA10">
-        <v>20.94</v>
+        <v>16.02</v>
       </c>
       <c r="AB10">
-        <v>8.539999999999999</v>
+        <v>615.38</v>
       </c>
       <c r="AC10">
-        <v>24.69</v>
+        <v>72.09</v>
       </c>
       <c r="AD10">
-        <v>5.93</v>
+        <v>7.76</v>
       </c>
       <c r="AE10">
-        <v>18.82</v>
+        <v>164.29</v>
       </c>
       <c r="AF10">
-        <v>11.84</v>
+        <v>147.06</v>
       </c>
       <c r="AG10">
-        <v>-6.17</v>
+        <v>-73.64</v>
       </c>
       <c r="AH10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AI10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AJ10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AK10">
-        <v>33.90367858123155</v>
+        <v>74.79684087478387</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -1743,49 +1734,49 @@
         <v>46</v>
       </c>
       <c r="B11">
-        <v>98.55072463768117</v>
+        <v>99.79253112033194</v>
       </c>
       <c r="C11">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="D11">
-        <v>85.31999999999999</v>
+        <v>14.72</v>
       </c>
       <c r="E11">
-        <v>1.24</v>
+        <v>2.52</v>
       </c>
       <c r="F11">
-        <v>-0.7777105688577521</v>
+        <v>2.491521328114704</v>
       </c>
       <c r="G11">
-        <v>1.77</v>
+        <v>2.61</v>
       </c>
       <c r="H11">
-        <v>-0.2490327407265248</v>
+        <v>1.608087839680521</v>
       </c>
       <c r="I11">
-        <v>84.63999786376954</v>
+        <v>14.84912509918213</v>
       </c>
       <c r="J11">
-        <v>81.74249992370605</v>
+        <v>14.24668750762939</v>
       </c>
       <c r="K11">
-        <v>77.52199981689454</v>
+        <v>13.75012500762939</v>
       </c>
       <c r="L11">
-        <v>63.53184991836548</v>
+        <v>10.81163749694824</v>
       </c>
       <c r="M11">
         <v>1.04</v>
       </c>
       <c r="N11">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="P11">
         <v>4</v>
       </c>
       <c r="Q11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -1794,58 +1785,58 @@
         <v>0</v>
       </c>
       <c r="T11">
-        <v>4.444444444444444</v>
+        <v>2.222222222222222</v>
       </c>
       <c r="U11" t="b">
         <v>1</v>
       </c>
       <c r="V11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11">
-        <v>39.02</v>
+        <v>5.46</v>
       </c>
       <c r="Y11">
-        <v>86.31999999999999</v>
+        <v>15.35</v>
       </c>
       <c r="Z11">
-        <v>89.89</v>
-      </c>
-      <c r="AA11">
-        <v>0.05</v>
+        <v>3.76</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>51</v>
       </c>
       <c r="AB11">
-        <v>0.68</v>
+        <v>58.13</v>
       </c>
       <c r="AC11">
-        <v>59.38</v>
+        <v>121.69</v>
       </c>
       <c r="AD11">
-        <v>3.88</v>
+        <v>8.77</v>
       </c>
       <c r="AE11">
-        <v>59.38</v>
+        <v>29.58</v>
       </c>
       <c r="AF11">
-        <v>-5.88</v>
+        <v>22.41</v>
       </c>
       <c r="AG11">
-        <v>6.25</v>
+        <v>39.76</v>
       </c>
       <c r="AH11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="AI11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AJ11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AK11">
-        <v>29.79500635297879</v>
+        <v>60.20736673698652</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -1853,46 +1844,46 @@
         <v>47</v>
       </c>
       <c r="B12">
-        <v>93.58178053830227</v>
+        <v>99.5850622406639</v>
       </c>
       <c r="C12">
-        <v>445</v>
+        <v>61</v>
       </c>
       <c r="D12">
-        <v>139.23</v>
+        <v>28.48</v>
       </c>
       <c r="E12">
-        <v>0.99</v>
+        <v>1.67</v>
       </c>
       <c r="F12">
-        <v>-1.094712159424771</v>
+        <v>0.8507995953574046</v>
       </c>
       <c r="G12">
-        <v>0.89</v>
+        <v>1.71</v>
       </c>
       <c r="H12">
-        <v>-1.590760160151068</v>
+        <v>0.2896135772935486</v>
       </c>
       <c r="I12">
-        <v>138.802001953125</v>
+        <v>28.1560001373291</v>
       </c>
       <c r="J12">
-        <v>136.1335021972656</v>
+        <v>27.85950002670288</v>
       </c>
       <c r="K12">
-        <v>131.0762010192871</v>
+        <v>27.57960010528565</v>
       </c>
       <c r="L12">
-        <v>115.3557001495361</v>
+        <v>22.3076000213623</v>
       </c>
       <c r="M12">
+        <v>1.01</v>
+      </c>
+      <c r="N12">
         <v>1.02</v>
       </c>
-      <c r="N12">
-        <v>1.06</v>
-      </c>
       <c r="P12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q12">
         <v>0</v>
@@ -1904,46 +1895,46 @@
         <v>0</v>
       </c>
       <c r="T12">
-        <v>2.777777777777778</v>
+        <v>0</v>
       </c>
       <c r="U12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V12" t="b">
         <v>1</v>
       </c>
       <c r="W12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12">
-        <v>82.62</v>
+        <v>12.19</v>
       </c>
       <c r="Y12">
-        <v>141.95</v>
+        <v>29.78</v>
       </c>
       <c r="Z12">
-        <v>10.74</v>
+        <v>8.24</v>
       </c>
       <c r="AA12">
-        <v>19.48</v>
+        <v>-171.36</v>
       </c>
       <c r="AB12">
-        <v>2.43</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="AC12">
-        <v>28.77</v>
+        <v>117.31</v>
       </c>
       <c r="AD12">
-        <v>23.63</v>
+        <v>5.01</v>
       </c>
       <c r="AE12">
-        <v>4.44</v>
+        <v>127.27</v>
       </c>
       <c r="AF12">
-        <v>12.5</v>
+        <v>-280.77</v>
       </c>
       <c r="AG12">
-        <v>9.59</v>
+        <v>83.33</v>
       </c>
       <c r="AH12" t="s">
         <v>60</v>
@@ -1952,10 +1943,10 @@
         <v>69</v>
       </c>
       <c r="AJ12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="AK12">
-        <v>27.18524975640464</v>
+        <v>58.89760856120674</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -1963,46 +1954,46 @@
         <v>48</v>
       </c>
       <c r="B13">
-        <v>98.34368530020704</v>
+        <v>96.88796680497926</v>
       </c>
       <c r="C13">
-        <v>364</v>
+        <v>447</v>
       </c>
       <c r="D13">
-        <v>34.94</v>
+        <v>69</v>
       </c>
       <c r="E13">
-        <v>1.87</v>
+        <v>1.21</v>
       </c>
       <c r="F13">
-        <v>0.02113343937113506</v>
+        <v>-0.03712040119360435</v>
       </c>
       <c r="G13">
-        <v>2.36</v>
+        <v>2.96</v>
       </c>
       <c r="H13">
-        <v>0.6505345063876576</v>
+        <v>2.120827830608789</v>
       </c>
       <c r="I13">
-        <v>34.70899963378906</v>
+        <v>69.17200012207032</v>
       </c>
       <c r="J13">
-        <v>32.98924989700318</v>
+        <v>69.32000007629395</v>
       </c>
       <c r="K13">
-        <v>31.19529998779297</v>
+        <v>67.27319999694824</v>
       </c>
       <c r="L13">
-        <v>23.57929993629456</v>
+        <v>53.90795000076294</v>
       </c>
       <c r="M13">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="N13">
-        <v>1.11</v>
+        <v>1.03</v>
       </c>
       <c r="P13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -2014,10 +2005,10 @@
         <v>0</v>
       </c>
       <c r="T13">
-        <v>0.5555555555555555</v>
+        <v>0</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="b">
         <v>1</v>
@@ -2026,46 +2017,46 @@
         <v>1</v>
       </c>
       <c r="X13">
-        <v>15.42</v>
+        <v>36.8</v>
       </c>
       <c r="Y13">
-        <v>35.4</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="Z13">
-        <v>2.02</v>
+        <v>3.2</v>
       </c>
       <c r="AA13">
-        <v>16.02</v>
+        <v>4.95</v>
       </c>
       <c r="AB13">
-        <v>615.38</v>
+        <v>50.47</v>
       </c>
       <c r="AC13">
-        <v>72.09</v>
+        <v>69.47</v>
       </c>
       <c r="AD13">
-        <v>7.76</v>
+        <v>-3</v>
       </c>
       <c r="AE13">
-        <v>164.29</v>
+        <v>69.23</v>
       </c>
       <c r="AF13">
-        <v>147.06</v>
+        <v>23.53</v>
       </c>
       <c r="AG13">
-        <v>-73.64</v>
+        <v>-29.77</v>
       </c>
       <c r="AH13" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="AI13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AJ13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="AK13">
-        <v>84.40318667870812</v>
+        <v>49.23213163427272</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -2073,46 +2064,46 @@
         <v>49</v>
       </c>
       <c r="B14">
-        <v>100</v>
+        <v>93.15352697095436</v>
       </c>
       <c r="C14">
-        <v>40</v>
+        <v>426</v>
       </c>
       <c r="D14">
-        <v>17.24</v>
+        <v>114.86</v>
       </c>
       <c r="E14">
-        <v>2.11</v>
+        <v>0.97</v>
       </c>
       <c r="F14">
-        <v>0.3254549663154727</v>
+        <v>-0.500383008089783</v>
       </c>
       <c r="G14">
-        <v>2.59</v>
+        <v>1.14</v>
       </c>
       <c r="H14">
-        <v>1.001213263737254</v>
+        <v>-0.5454201222182009</v>
       </c>
       <c r="I14">
-        <v>17.36625022888184</v>
+        <v>114.9119995117187</v>
       </c>
       <c r="J14">
-        <v>16.37834391593933</v>
+        <v>114.3965000152588</v>
       </c>
       <c r="K14">
-        <v>15.22338756561279</v>
+        <v>110.0283999633789</v>
       </c>
       <c r="L14">
-        <v>11.65565313816071</v>
+        <v>94.44595008850098</v>
       </c>
       <c r="M14">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="N14">
-        <v>1.14</v>
+        <v>1.04</v>
       </c>
       <c r="P14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q14">
         <v>0</v>
@@ -2124,278 +2115,58 @@
         <v>0</v>
       </c>
       <c r="T14">
-        <v>2.222222222222222</v>
+        <v>0</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X14">
-        <v>5.8</v>
+        <v>69.53</v>
       </c>
       <c r="Y14">
-        <v>17.8</v>
+        <v>117.92</v>
       </c>
       <c r="Z14">
-        <v>3.76</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>53</v>
+        <v>8.84</v>
+      </c>
+      <c r="AA14">
+        <v>17.13</v>
       </c>
       <c r="AB14">
-        <v>58.13</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="AC14">
-        <v>121.69</v>
+        <v>75.70999999999999</v>
       </c>
       <c r="AD14">
-        <v>8.77</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="AE14">
-        <v>29.58</v>
+        <v>-10.22</v>
       </c>
       <c r="AF14">
-        <v>22.41</v>
+        <v>7.87</v>
       </c>
       <c r="AG14">
-        <v>39.76</v>
+        <v>81.43000000000001</v>
       </c>
       <c r="AH14" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="AI14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AJ14" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AK14">
-        <v>69.64822775975573</v>
-      </c>
-    </row>
-    <row r="15" spans="1:37">
-      <c r="A15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15">
-        <v>96.8944099378882</v>
-      </c>
-      <c r="C15">
-        <v>472</v>
-      </c>
-      <c r="D15">
-        <v>76.53</v>
-      </c>
-      <c r="E15">
-        <v>3.45</v>
-      </c>
-      <c r="F15">
-        <v>2.024583491754693</v>
-      </c>
-      <c r="G15">
-        <v>3.4</v>
-      </c>
-      <c r="H15">
-        <v>2.236212365707573</v>
-      </c>
-      <c r="I15">
-        <v>77.33799896240234</v>
-      </c>
-      <c r="J15">
-        <v>74.92150039672852</v>
-      </c>
-      <c r="K15">
-        <v>71.85200012207031</v>
-      </c>
-      <c r="L15">
-        <v>57.28055006027222</v>
-      </c>
-      <c r="M15">
-        <v>1.03</v>
-      </c>
-      <c r="N15">
-        <v>1.08</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>0</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-      <c r="T15">
-        <v>0</v>
-      </c>
-      <c r="U15" t="b">
-        <v>0</v>
-      </c>
-      <c r="V15" t="b">
-        <v>1</v>
-      </c>
-      <c r="W15" t="b">
-        <v>1</v>
-      </c>
-      <c r="X15">
-        <v>38.43</v>
-      </c>
-      <c r="Y15">
-        <v>78.65000000000001</v>
-      </c>
-      <c r="Z15">
-        <v>3.2</v>
-      </c>
-      <c r="AA15">
-        <v>4.95</v>
-      </c>
-      <c r="AB15">
-        <v>50.47</v>
-      </c>
-      <c r="AC15">
-        <v>69.47</v>
-      </c>
-      <c r="AD15">
-        <v>-3</v>
-      </c>
-      <c r="AE15">
-        <v>69.23</v>
-      </c>
-      <c r="AF15">
-        <v>23.53</v>
-      </c>
-      <c r="AG15">
-        <v>-29.77</v>
-      </c>
-      <c r="AH15" t="s">
-        <v>62</v>
-      </c>
-      <c r="AI15" t="s">
-        <v>68</v>
-      </c>
-      <c r="AJ15" t="s">
-        <v>83</v>
-      </c>
-      <c r="AK15">
-        <v>60.48679655466721</v>
-      </c>
-    </row>
-    <row r="16" spans="1:37">
-      <c r="A16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16">
-        <v>93.7888198757764</v>
-      </c>
-      <c r="C16">
-        <v>481</v>
-      </c>
-      <c r="D16">
-        <v>179.02</v>
-      </c>
-      <c r="E16">
-        <v>3.12</v>
-      </c>
-      <c r="F16">
-        <v>1.606141392206228</v>
-      </c>
-      <c r="G16">
-        <v>2.04</v>
-      </c>
-      <c r="H16">
-        <v>0.1626336265969148</v>
-      </c>
-      <c r="I16">
-        <v>179.5426635742188</v>
-      </c>
-      <c r="J16">
-        <v>173.3099998474121</v>
-      </c>
-      <c r="K16">
-        <v>151.9654656982422</v>
-      </c>
-      <c r="L16">
-        <v>124.7444332885742</v>
-      </c>
-      <c r="M16">
-        <v>1.04</v>
-      </c>
-      <c r="N16">
-        <v>1.18</v>
-      </c>
-      <c r="P16">
-        <v>0</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
-        <v>3</v>
-      </c>
-      <c r="T16">
-        <v>5</v>
-      </c>
-      <c r="U16" t="b">
-        <v>0</v>
-      </c>
-      <c r="V16" t="b">
-        <v>0</v>
-      </c>
-      <c r="W16" t="b">
-        <v>1</v>
-      </c>
-      <c r="X16">
-        <v>86.33</v>
-      </c>
-      <c r="Y16">
-        <v>190</v>
-      </c>
-      <c r="Z16">
-        <v>3.51</v>
-      </c>
-      <c r="AA16">
-        <v>104.17</v>
-      </c>
-      <c r="AB16">
-        <v>60.37</v>
-      </c>
-      <c r="AC16">
-        <v>30.46</v>
-      </c>
-      <c r="AD16">
-        <v>23.43</v>
-      </c>
-      <c r="AE16">
-        <v>-24.52</v>
-      </c>
-      <c r="AF16">
-        <v>62.79</v>
-      </c>
-      <c r="AG16">
-        <v>6.17</v>
-      </c>
-      <c r="AH16" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI16" t="s">
-        <v>70</v>
-      </c>
-      <c r="AJ16" t="s">
-        <v>84</v>
-      </c>
-      <c r="AK16">
-        <v>56.16785986374261</v>
+        <v>32.50442284193593</v>
       </c>
     </row>
   </sheetData>

</xml_diff>